<commit_message>
feat(minor-hotels): ground Palm crescent BPs — aspirational → solid
Snap 3 Minor property POIs to gold gazetteer jetty BPs, scope 13 crescent
boarding points to dubai-uae__palm-jumeirah-crescent-inner, un-quarantine
3 captive routes, and upgrade Palm market render from amber to solid.

- Add ground_palm_crescent.py + seal lane step 2/4
- City brief → active_geometry; partner journeys bound to bp-* nodes
- Add rn-b0d5e6498ee4 to uae-luxury corridors for Class A cascade
- Palm cluster status: economics_ready (3 corridors, $3.75M floor)
</commit_message>
<xml_diff>
--- a/finance/_refresh_minor-hotels.xlsx
+++ b/finance/_refresh_minor-hotels.xlsx
@@ -3315,11 +3315,11 @@
       </c>
       <c r="C9" s="30" t="inlineStr">
         <is>
-          <t>Dubai Harbour Marina → Nikki Beach Resort Pearl Jumeirah Jetty</t>
+          <t>Dubai Harbour Marina → Anantara The Palm Dubai Jetty</t>
         </is>
       </c>
       <c r="D9" s="31" t="n">
-        <v>11.9</v>
+        <v>3.4</v>
       </c>
       <c r="E9" s="26" t="n">
         <v>150</v>

</xml_diff>

<commit_message>
feat(minor-hotels): cascade Class A/B journeys into economics sidecar
Add 5 grounded rn-* corridors to phuket/bali parent markets and
TIER1_CORRIDOR_ROUTES; fix sidecar to merge agg-minor-hotels when
corridors-minor-hotels.json is scoped. All 12 Tier-1 journeys now
economics_status: bound with per-route sidecar records.

Market headline floors unchanged ($4.38M / $0.63M / $3.75M).
</commit_message>
<xml_diff>
--- a/finance/_refresh_minor-hotels.xlsx
+++ b/finance/_refresh_minor-hotels.xlsx
@@ -45,8 +45,8 @@
     <definedName name="load_sel">'Assumptions'!$B$39</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$40</definedName>
     <definedName name="country_opex">'Country opex'!$A$4:$G$6</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$17</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$17</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$23</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -60,7 +60,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,15 +108,6 @@
     <font>
       <color rgb="009C4500"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="9">
@@ -188,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -325,12 +316,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1973,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY19"/>
+  <dimension ref="A1:AY23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2320,11 +2305,11 @@
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>Bali (Benoa / Sanur) → Nusa Penida / Lembongan</t>
+          <t>Sanur Beach Fast Boat Terminal → GoBoat.id - Nelayan Beach Canggu</t>
         </is>
       </c>
       <c r="D4" s="31" t="n">
-        <v>13.5</v>
+        <v>7.6</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>85</v>
@@ -2439,7 +2424,7 @@
         <v/>
       </c>
       <c r="AG4" s="31" t="n">
-        <v>8756</v>
+        <v>2919</v>
       </c>
       <c r="AH4" s="32" t="inlineStr">
         <is>
@@ -2509,24 +2494,24 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Bali</t>
         </is>
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Phuket (Royal Phuket Marina) → Phang Nga Bay / James Bond Island</t>
+          <t>Bali Marina (Benoa) → Six Senses Uluwatu</t>
         </is>
       </c>
       <c r="D5" s="31" t="n">
-        <v>20</v>
+        <v>7.7</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="F5" s="32" t="inlineStr">
         <is>
@@ -2638,7 +2623,7 @@
         <v/>
       </c>
       <c r="AG5" s="31" t="n">
-        <v>17182</v>
+        <v>2919</v>
       </c>
       <c r="AH5" s="32" t="inlineStr">
         <is>
@@ -2696,36 +2681,36 @@
       </c>
       <c r="AX5" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+          <t>minor-hotels/bali grounded floor</t>
         </is>
       </c>
       <c r="AY5" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+          <t>minor-hotels/bali grounded floor</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Phuket</t>
+          <t>Bali</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>Phuket → Krabi (Ao Nang)</t>
+          <t>Bali (Benoa / Sanur) → Nusa Penida / Lembongan</t>
         </is>
       </c>
       <c r="D6" s="31" t="n">
-        <v>40</v>
+        <v>13.5</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="F6" s="32" t="inlineStr">
         <is>
@@ -2837,7 +2822,7 @@
         <v/>
       </c>
       <c r="AG6" s="31" t="n">
-        <v>17182</v>
+        <v>2918</v>
       </c>
       <c r="AH6" s="32" t="inlineStr">
         <is>
@@ -2895,36 +2880,36 @@
       </c>
       <c r="AX6" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+          <t>minor-hotels/bali grounded floor</t>
         </is>
       </c>
       <c r="AY6" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+          <t>minor-hotels/bali grounded floor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Palm Jumeirah</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>Palm Jumeirah Marina West → Atlantis The Palm Jetty</t>
+          <t>Ao Po Grand Marina → Anantara Layan Phuket Beach Jetty</t>
         </is>
       </c>
       <c r="D7" s="31" t="n">
-        <v>1.3</v>
+        <v>9.6</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F7" s="32" t="inlineStr">
         <is>
@@ -3036,7 +3021,7 @@
         <v/>
       </c>
       <c r="AG7" s="31" t="n">
-        <v>13897</v>
+        <v>8591</v>
       </c>
       <c r="AH7" s="32" t="inlineStr">
         <is>
@@ -3094,36 +3079,36 @@
       </c>
       <c r="AX7" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/palm-jumeirah grounded floor</t>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
         </is>
       </c>
       <c r="AY7" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/palm-jumeirah grounded floor</t>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Palm Jumeirah</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>Dubai Harbour Marina → Palm Jumeirah Marina West</t>
+          <t>Rassada Pier (Phuket Deep Sea Port) → Manoh Pier (Koh Yao Yai)</t>
         </is>
       </c>
       <c r="D8" s="31" t="n">
-        <v>2.1</v>
+        <v>16.9</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F8" s="32" t="inlineStr">
         <is>
@@ -3235,7 +3220,7 @@
         <v/>
       </c>
       <c r="AG8" s="31" t="n">
-        <v>13897</v>
+        <v>8591</v>
       </c>
       <c r="AH8" s="32" t="inlineStr">
         <is>
@@ -3293,36 +3278,36 @@
       </c>
       <c r="AX8" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/palm-jumeirah grounded floor</t>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
         </is>
       </c>
       <c r="AY8" s="44" t="inlineStr">
         <is>
-          <t>minor-hotels/palm-jumeirah grounded floor</t>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Palm Jumeirah</t>
+          <t>Phuket</t>
         </is>
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C9" s="30" t="inlineStr">
         <is>
-          <t>Dubai Harbour Marina → Anantara The Palm Dubai Jetty</t>
+          <t>Phuket (Royal Phuket Marina) → Phang Nga Bay / James Bond Island</t>
         </is>
       </c>
       <c r="D9" s="31" t="n">
-        <v>3.4</v>
+        <v>20</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F9" s="32" t="inlineStr">
         <is>
@@ -3434,7 +3419,7 @@
         <v/>
       </c>
       <c r="AG9" s="31" t="n">
-        <v>13897</v>
+        <v>8591</v>
       </c>
       <c r="AH9" s="32" t="inlineStr">
         <is>
@@ -3492,179 +3477,1361 @@
       </c>
       <c r="AX9" s="44" t="inlineStr">
         <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+      <c r="AY9" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>Phuket → Phi Phi (Tonsai)</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="33">
+        <f>60*D10/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J10" s="33">
+        <f>I10+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K10" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J10,1))</f>
+        <v/>
+      </c>
+      <c r="L10" s="34">
+        <f>ROUND(365*mech_uptime*H10,0)</f>
+        <v/>
+      </c>
+      <c r="M10" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N10" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O10" s="34">
+        <f>ROUND(K10*L10*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q10" s="36">
+        <f>pax_cap*P10</f>
+        <v/>
+      </c>
+      <c r="R10" s="34">
+        <f>Q10*O10</f>
+        <v/>
+      </c>
+      <c r="S10" s="37">
+        <f>E10*discount</f>
+        <v/>
+      </c>
+      <c r="T10" s="38">
+        <f>S10*R10</f>
+        <v/>
+      </c>
+      <c r="U10" s="38">
+        <f>(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V10" s="38">
+        <f>VLOOKUP(B10,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W10" s="38">
+        <f>VLOOKUP(B10,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X10" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y10" s="38">
+        <f>VLOOKUP(B10,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z10" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA10" s="38">
+        <f>U10+V10+W10+X10+Y10+Z10</f>
+        <v/>
+      </c>
+      <c r="AB10" s="38">
+        <f>VLOOKUP(B10,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC10" s="38">
+        <f>T10-AA10</f>
+        <v/>
+      </c>
+      <c r="AD10" s="35">
+        <f>IF(T10=0,"",AC10/T10)</f>
+        <v/>
+      </c>
+      <c r="AE10" s="36">
+        <f>IF(AC10&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/AC10)</f>
+        <v/>
+      </c>
+      <c r="AF10" s="33">
+        <f>((D10*O10/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG10" s="31" t="n">
+        <v>8591</v>
+      </c>
+      <c r="AH10" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI10" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ10" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK10" s="34">
+        <f>IF(AG10="","",AG10*AJ10)</f>
+        <v/>
+      </c>
+      <c r="AL10" s="34">
+        <f>IF(OR(AG10="",R10=0),"",MIN(IF(AT10="",9.9E+99,AT10),FLOOR(AK10/R10,1)))</f>
+        <v/>
+      </c>
+      <c r="AM10" s="38">
+        <f>IF(AL10="","",AL10*T10)</f>
+        <v/>
+      </c>
+      <c r="AN10" s="36">
+        <f>IF(OR(AG10="",R10=0),"",MIN(IF(AT10="",9.9E+99,AT10),AK10/R10))</f>
+        <v/>
+      </c>
+      <c r="AO10" s="38">
+        <f>IF(AN10="","",AN10*T10)</f>
+        <v/>
+      </c>
+      <c r="AP10" s="40" t="n"/>
+      <c r="AQ10" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR10" s="41" t="n"/>
+      <c r="AS10" s="41" t="n"/>
+      <c r="AT10" s="42" t="n"/>
+      <c r="AU10" s="43">
+        <f>IF(((S10*pax_cap*load_thin*ROUND(K10*L10*revleg_thin,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_thin,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_thin*ROUND(K10*L10*revleg_thin,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_thin,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AV10" s="43">
+        <f>IF(((S10*pax_cap*load_mid*ROUND(K10*L10*revleg_mid,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_mid,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_mid*ROUND(K10*L10*revleg_mid,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_mid,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AW10" s="43">
+        <f>IF(((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AX10" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+      <c r="AY10" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>Manoh Pier (Koh Yao Yai) → Thap Lamu Pier (Similan Gateway)</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="E11" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="33">
+        <f>60*D11/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J11" s="33">
+        <f>I11+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K11" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J11,1))</f>
+        <v/>
+      </c>
+      <c r="L11" s="34">
+        <f>ROUND(365*mech_uptime*H11,0)</f>
+        <v/>
+      </c>
+      <c r="M11" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N11" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O11" s="34">
+        <f>ROUND(K11*L11*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q11" s="36">
+        <f>pax_cap*P11</f>
+        <v/>
+      </c>
+      <c r="R11" s="34">
+        <f>Q11*O11</f>
+        <v/>
+      </c>
+      <c r="S11" s="37">
+        <f>E11*discount</f>
+        <v/>
+      </c>
+      <c r="T11" s="38">
+        <f>S11*R11</f>
+        <v/>
+      </c>
+      <c r="U11" s="38">
+        <f>(battery/range_nm)*D11*O11*VLOOKUP(B11,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V11" s="38">
+        <f>VLOOKUP(B11,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W11" s="38">
+        <f>VLOOKUP(B11,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X11" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y11" s="38">
+        <f>VLOOKUP(B11,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z11" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA11" s="38">
+        <f>U11+V11+W11+X11+Y11+Z11</f>
+        <v/>
+      </c>
+      <c r="AB11" s="38">
+        <f>VLOOKUP(B11,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC11" s="38">
+        <f>T11-AA11</f>
+        <v/>
+      </c>
+      <c r="AD11" s="35">
+        <f>IF(T11=0,"",AC11/T11)</f>
+        <v/>
+      </c>
+      <c r="AE11" s="36">
+        <f>IF(AC11&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/AC11)</f>
+        <v/>
+      </c>
+      <c r="AF11" s="33">
+        <f>((D11*O11/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D11*O11*VLOOKUP(B11,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG11" s="31" t="n">
+        <v>8591</v>
+      </c>
+      <c r="AH11" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI11" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ11" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK11" s="34">
+        <f>IF(AG11="","",AG11*AJ11)</f>
+        <v/>
+      </c>
+      <c r="AL11" s="34">
+        <f>IF(OR(AG11="",R11=0),"",MIN(IF(AT11="",9.9E+99,AT11),FLOOR(AK11/R11,1)))</f>
+        <v/>
+      </c>
+      <c r="AM11" s="38">
+        <f>IF(AL11="","",AL11*T11)</f>
+        <v/>
+      </c>
+      <c r="AN11" s="36">
+        <f>IF(OR(AG11="",R11=0),"",MIN(IF(AT11="",9.9E+99,AT11),AK11/R11))</f>
+        <v/>
+      </c>
+      <c r="AO11" s="38">
+        <f>IF(AN11="","",AN11*T11)</f>
+        <v/>
+      </c>
+      <c r="AP11" s="40" t="n"/>
+      <c r="AQ11" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR11" s="41" t="n"/>
+      <c r="AS11" s="41" t="n"/>
+      <c r="AT11" s="42" t="n"/>
+      <c r="AU11" s="43">
+        <f>IF(((S11*pax_cap*load_thin*ROUND(K11*L11*revleg_thin,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_thin,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_thin*ROUND(K11*L11*revleg_thin,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_thin,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
+        <v/>
+      </c>
+      <c r="AV11" s="43">
+        <f>IF(((S11*pax_cap*load_mid*ROUND(K11*L11*revleg_mid,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_mid,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_mid*ROUND(K11*L11*revleg_mid,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_mid,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
+        <v/>
+      </c>
+      <c r="AW11" s="43">
+        <f>IF(((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
+        <v/>
+      </c>
+      <c r="AX11" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+      <c r="AY11" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Phuket</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Phuket → Krabi (Ao Nang)</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="33">
+        <f>60*D12/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J12" s="33">
+        <f>I12+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K12" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J12,1))</f>
+        <v/>
+      </c>
+      <c r="L12" s="34">
+        <f>ROUND(365*mech_uptime*H12,0)</f>
+        <v/>
+      </c>
+      <c r="M12" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N12" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O12" s="34">
+        <f>ROUND(K12*L12*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q12" s="36">
+        <f>pax_cap*P12</f>
+        <v/>
+      </c>
+      <c r="R12" s="34">
+        <f>Q12*O12</f>
+        <v/>
+      </c>
+      <c r="S12" s="37">
+        <f>E12*discount</f>
+        <v/>
+      </c>
+      <c r="T12" s="38">
+        <f>S12*R12</f>
+        <v/>
+      </c>
+      <c r="U12" s="38">
+        <f>(battery/range_nm)*D12*O12*VLOOKUP(B12,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V12" s="38">
+        <f>VLOOKUP(B12,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W12" s="38">
+        <f>VLOOKUP(B12,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X12" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y12" s="38">
+        <f>VLOOKUP(B12,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z12" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA12" s="38">
+        <f>U12+V12+W12+X12+Y12+Z12</f>
+        <v/>
+      </c>
+      <c r="AB12" s="38">
+        <f>VLOOKUP(B12,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC12" s="38">
+        <f>T12-AA12</f>
+        <v/>
+      </c>
+      <c r="AD12" s="35">
+        <f>IF(T12=0,"",AC12/T12)</f>
+        <v/>
+      </c>
+      <c r="AE12" s="36">
+        <f>IF(AC12&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/AC12)</f>
+        <v/>
+      </c>
+      <c r="AF12" s="33">
+        <f>((D12*O12/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D12*O12*VLOOKUP(B12,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG12" s="31" t="n">
+        <v>8590</v>
+      </c>
+      <c r="AH12" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI12" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ12" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK12" s="34">
+        <f>IF(AG12="","",AG12*AJ12)</f>
+        <v/>
+      </c>
+      <c r="AL12" s="34">
+        <f>IF(OR(AG12="",R12=0),"",MIN(IF(AT12="",9.9E+99,AT12),FLOOR(AK12/R12,1)))</f>
+        <v/>
+      </c>
+      <c r="AM12" s="38">
+        <f>IF(AL12="","",AL12*T12)</f>
+        <v/>
+      </c>
+      <c r="AN12" s="36">
+        <f>IF(OR(AG12="",R12=0),"",MIN(IF(AT12="",9.9E+99,AT12),AK12/R12))</f>
+        <v/>
+      </c>
+      <c r="AO12" s="38">
+        <f>IF(AN12="","",AN12*T12)</f>
+        <v/>
+      </c>
+      <c r="AP12" s="40" t="n"/>
+      <c r="AQ12" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR12" s="41" t="n"/>
+      <c r="AS12" s="41" t="n"/>
+      <c r="AT12" s="42" t="n"/>
+      <c r="AU12" s="43">
+        <f>IF(((S12*pax_cap*load_thin*ROUND(K12*L12*revleg_thin,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_thin,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((S12*pax_cap*load_thin*ROUND(K12*L12*revleg_thin,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_thin,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12)))</f>
+        <v/>
+      </c>
+      <c r="AV12" s="43">
+        <f>IF(((S12*pax_cap*load_mid*ROUND(K12*L12*revleg_mid,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_mid,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((S12*pax_cap*load_mid*ROUND(K12*L12*revleg_mid,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_mid,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12)))</f>
+        <v/>
+      </c>
+      <c r="AW12" s="43">
+        <f>IF(((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((S12*pax_cap*load_full*ROUND(K12*L12*revleg_full,0))-(((battery/range_nm)*D12*ROUND(K12*L12*revleg_full,0)*VLOOKUP(B12,country_opex,3,FALSE))+V12+W12+X12+Y12+Z12)))</f>
+        <v/>
+      </c>
+      <c r="AX12" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+      <c r="AY12" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/phuket-phang-nga grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Palm Jumeirah</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Palm Jumeirah Marina West → Atlantis The Palm Jetty</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E13" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="33">
+        <f>60*D13/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J13" s="33">
+        <f>I13+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K13" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J13,1))</f>
+        <v/>
+      </c>
+      <c r="L13" s="34">
+        <f>ROUND(365*mech_uptime*H13,0)</f>
+        <v/>
+      </c>
+      <c r="M13" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N13" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O13" s="34">
+        <f>ROUND(K13*L13*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P13" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q13" s="36">
+        <f>pax_cap*P13</f>
+        <v/>
+      </c>
+      <c r="R13" s="34">
+        <f>Q13*O13</f>
+        <v/>
+      </c>
+      <c r="S13" s="37">
+        <f>E13*discount</f>
+        <v/>
+      </c>
+      <c r="T13" s="38">
+        <f>S13*R13</f>
+        <v/>
+      </c>
+      <c r="U13" s="38">
+        <f>(battery/range_nm)*D13*O13*VLOOKUP(B13,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V13" s="38">
+        <f>VLOOKUP(B13,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W13" s="38">
+        <f>VLOOKUP(B13,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X13" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y13" s="38">
+        <f>VLOOKUP(B13,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z13" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA13" s="38">
+        <f>U13+V13+W13+X13+Y13+Z13</f>
+        <v/>
+      </c>
+      <c r="AB13" s="38">
+        <f>VLOOKUP(B13,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC13" s="38">
+        <f>T13-AA13</f>
+        <v/>
+      </c>
+      <c r="AD13" s="35">
+        <f>IF(T13=0,"",AC13/T13)</f>
+        <v/>
+      </c>
+      <c r="AE13" s="36">
+        <f>IF(AC13&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/AC13)</f>
+        <v/>
+      </c>
+      <c r="AF13" s="33">
+        <f>((D13*O13/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D13*O13*VLOOKUP(B13,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG13" s="31" t="n">
+        <v>13897</v>
+      </c>
+      <c r="AH13" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI13" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ13" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK13" s="34">
+        <f>IF(AG13="","",AG13*AJ13)</f>
+        <v/>
+      </c>
+      <c r="AL13" s="34">
+        <f>IF(OR(AG13="",R13=0),"",MIN(IF(AT13="",9.9E+99,AT13),FLOOR(AK13/R13,1)))</f>
+        <v/>
+      </c>
+      <c r="AM13" s="38">
+        <f>IF(AL13="","",AL13*T13)</f>
+        <v/>
+      </c>
+      <c r="AN13" s="36">
+        <f>IF(OR(AG13="",R13=0),"",MIN(IF(AT13="",9.9E+99,AT13),AK13/R13))</f>
+        <v/>
+      </c>
+      <c r="AO13" s="38">
+        <f>IF(AN13="","",AN13*T13)</f>
+        <v/>
+      </c>
+      <c r="AP13" s="40" t="n"/>
+      <c r="AQ13" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR13" s="41" t="n"/>
+      <c r="AS13" s="41" t="n"/>
+      <c r="AT13" s="42" t="n"/>
+      <c r="AU13" s="43">
+        <f>IF(((S13*pax_cap*load_thin*ROUND(K13*L13*revleg_thin,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_thin,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((S13*pax_cap*load_thin*ROUND(K13*L13*revleg_thin,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_thin,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13)))</f>
+        <v/>
+      </c>
+      <c r="AV13" s="43">
+        <f>IF(((S13*pax_cap*load_mid*ROUND(K13*L13*revleg_mid,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_mid,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((S13*pax_cap*load_mid*ROUND(K13*L13*revleg_mid,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_mid,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13)))</f>
+        <v/>
+      </c>
+      <c r="AW13" s="43">
+        <f>IF(((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13)))</f>
+        <v/>
+      </c>
+      <c r="AX13" s="44" t="inlineStr">
+        <is>
           <t>minor-hotels/palm-jumeirah grounded floor</t>
         </is>
       </c>
-      <c r="AY9" s="44" t="inlineStr">
+      <c r="AY13" s="44" t="inlineStr">
         <is>
           <t>minor-hotels/palm-jumeirah grounded floor</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="45" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Palm Jumeirah</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Dubai Harbour Marina → Palm Jumeirah Marina West</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E14" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="33">
+        <f>60*D14/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J14" s="33">
+        <f>I14+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K14" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J14,1))</f>
+        <v/>
+      </c>
+      <c r="L14" s="34">
+        <f>ROUND(365*mech_uptime*H14,0)</f>
+        <v/>
+      </c>
+      <c r="M14" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N14" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O14" s="34">
+        <f>ROUND(K14*L14*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q14" s="36">
+        <f>pax_cap*P14</f>
+        <v/>
+      </c>
+      <c r="R14" s="34">
+        <f>Q14*O14</f>
+        <v/>
+      </c>
+      <c r="S14" s="37">
+        <f>E14*discount</f>
+        <v/>
+      </c>
+      <c r="T14" s="38">
+        <f>S14*R14</f>
+        <v/>
+      </c>
+      <c r="U14" s="38">
+        <f>(battery/range_nm)*D14*O14*VLOOKUP(B14,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V14" s="38">
+        <f>VLOOKUP(B14,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W14" s="38">
+        <f>VLOOKUP(B14,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X14" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y14" s="38">
+        <f>VLOOKUP(B14,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z14" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA14" s="38">
+        <f>U14+V14+W14+X14+Y14+Z14</f>
+        <v/>
+      </c>
+      <c r="AB14" s="38">
+        <f>VLOOKUP(B14,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC14" s="38">
+        <f>T14-AA14</f>
+        <v/>
+      </c>
+      <c r="AD14" s="35">
+        <f>IF(T14=0,"",AC14/T14)</f>
+        <v/>
+      </c>
+      <c r="AE14" s="36">
+        <f>IF(AC14&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/AC14)</f>
+        <v/>
+      </c>
+      <c r="AF14" s="33">
+        <f>((D14*O14/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D14*O14*VLOOKUP(B14,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG14" s="31" t="n">
+        <v>13897</v>
+      </c>
+      <c r="AH14" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI14" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ14" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK14" s="34">
+        <f>IF(AG14="","",AG14*AJ14)</f>
+        <v/>
+      </c>
+      <c r="AL14" s="34">
+        <f>IF(OR(AG14="",R14=0),"",MIN(IF(AT14="",9.9E+99,AT14),FLOOR(AK14/R14,1)))</f>
+        <v/>
+      </c>
+      <c r="AM14" s="38">
+        <f>IF(AL14="","",AL14*T14)</f>
+        <v/>
+      </c>
+      <c r="AN14" s="36">
+        <f>IF(OR(AG14="",R14=0),"",MIN(IF(AT14="",9.9E+99,AT14),AK14/R14))</f>
+        <v/>
+      </c>
+      <c r="AO14" s="38">
+        <f>IF(AN14="","",AN14*T14)</f>
+        <v/>
+      </c>
+      <c r="AP14" s="40" t="n"/>
+      <c r="AQ14" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR14" s="41" t="n"/>
+      <c r="AS14" s="41" t="n"/>
+      <c r="AT14" s="42" t="n"/>
+      <c r="AU14" s="43">
+        <f>IF(((S14*pax_cap*load_thin*ROUND(K14*L14*revleg_thin,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_thin,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_thin*ROUND(K14*L14*revleg_thin,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_thin,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
+        <v/>
+      </c>
+      <c r="AV14" s="43">
+        <f>IF(((S14*pax_cap*load_mid*ROUND(K14*L14*revleg_mid,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_mid,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_mid*ROUND(K14*L14*revleg_mid,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_mid,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
+        <v/>
+      </c>
+      <c r="AW14" s="43">
+        <f>IF(((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
+        <v/>
+      </c>
+      <c r="AX14" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/palm-jumeirah grounded floor</t>
+        </is>
+      </c>
+      <c r="AY14" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/palm-jumeirah grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Palm Jumeirah</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Dubai Harbour Marina → Anantara The Palm Dubai Jetty</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E15" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G15" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="33">
+        <f>60*D15/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J15" s="33">
+        <f>I15+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K15" s="34">
+        <f>MIN(15,FLOOR(60*service_hr/J15,1))</f>
+        <v/>
+      </c>
+      <c r="L15" s="34">
+        <f>ROUND(365*mech_uptime*H15,0)</f>
+        <v/>
+      </c>
+      <c r="M15" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N15" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O15" s="34">
+        <f>ROUND(K15*L15*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P15" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q15" s="36">
+        <f>pax_cap*P15</f>
+        <v/>
+      </c>
+      <c r="R15" s="34">
+        <f>Q15*O15</f>
+        <v/>
+      </c>
+      <c r="S15" s="37">
+        <f>E15*discount</f>
+        <v/>
+      </c>
+      <c r="T15" s="38">
+        <f>S15*R15</f>
+        <v/>
+      </c>
+      <c r="U15" s="38">
+        <f>(battery/range_nm)*D15*O15*VLOOKUP(B15,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V15" s="38">
+        <f>VLOOKUP(B15,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W15" s="38">
+        <f>VLOOKUP(B15,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X15" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y15" s="38">
+        <f>VLOOKUP(B15,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z15" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA15" s="38">
+        <f>U15+V15+W15+X15+Y15+Z15</f>
+        <v/>
+      </c>
+      <c r="AB15" s="38">
+        <f>VLOOKUP(B15,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC15" s="38">
+        <f>T15-AA15</f>
+        <v/>
+      </c>
+      <c r="AD15" s="35">
+        <f>IF(T15=0,"",AC15/T15)</f>
+        <v/>
+      </c>
+      <c r="AE15" s="36">
+        <f>IF(AC15&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/AC15)</f>
+        <v/>
+      </c>
+      <c r="AF15" s="33">
+        <f>((D15*O15/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D15*O15*VLOOKUP(B15,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG15" s="31" t="n">
+        <v>13897</v>
+      </c>
+      <c r="AH15" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="AI15" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="AJ15" s="39" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AK15" s="34">
+        <f>IF(AG15="","",AG15*AJ15)</f>
+        <v/>
+      </c>
+      <c r="AL15" s="34">
+        <f>IF(OR(AG15="",R15=0),"",MIN(IF(AT15="",9.9E+99,AT15),FLOOR(AK15/R15,1)))</f>
+        <v/>
+      </c>
+      <c r="AM15" s="38">
+        <f>IF(AL15="","",AL15*T15)</f>
+        <v/>
+      </c>
+      <c r="AN15" s="36">
+        <f>IF(OR(AG15="",R15=0),"",MIN(IF(AT15="",9.9E+99,AT15),AK15/R15))</f>
+        <v/>
+      </c>
+      <c r="AO15" s="38">
+        <f>IF(AN15="","",AN15*T15)</f>
+        <v/>
+      </c>
+      <c r="AP15" s="40" t="n"/>
+      <c r="AQ15" s="32" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="AR15" s="41" t="n"/>
+      <c r="AS15" s="41" t="n"/>
+      <c r="AT15" s="42" t="n"/>
+      <c r="AU15" s="43">
+        <f>IF(((S15*pax_cap*load_thin*ROUND(K15*L15*revleg_thin,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_thin,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15))&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/((S15*pax_cap*load_thin*ROUND(K15*L15*revleg_thin,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_thin,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15)))</f>
+        <v/>
+      </c>
+      <c r="AV15" s="43">
+        <f>IF(((S15*pax_cap*load_mid*ROUND(K15*L15*revleg_mid,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_mid,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15))&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/((S15*pax_cap*load_mid*ROUND(K15*L15*revleg_mid,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_mid,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15)))</f>
+        <v/>
+      </c>
+      <c r="AW15" s="43">
+        <f>IF(((S15*pax_cap*load_full*ROUND(K15*L15*revleg_full,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_full,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15))&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/((S15*pax_cap*load_full*ROUND(K15*L15*revleg_full,0))-(((battery/range_nm)*D15*ROUND(K15*L15*revleg_full,0)*VLOOKUP(B15,country_opex,3,FALSE))+V15+W15+X15+Y15+Z15)))</f>
+        <v/>
+      </c>
+      <c r="AX15" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/palm-jumeirah grounded floor</t>
+        </is>
+      </c>
+      <c r="AY15" s="44" t="inlineStr">
+        <is>
+          <t>minor-hotels/palm-jumeirah grounded floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="45" t="inlineStr">
         <is>
           <t>TOTAL / median</t>
         </is>
       </c>
-      <c r="T10" s="46">
-        <f>SUM(T4:T9)</f>
-        <v/>
-      </c>
-      <c r="AC10" s="46">
-        <f>SUM(AC4:AC9)</f>
-        <v/>
-      </c>
-      <c r="AD10" s="47">
-        <f>IF(T10=0,"",AC10/T10)</f>
-        <v/>
-      </c>
-      <c r="AL10" s="48">
-        <f>SUM(AL4:AL9)</f>
-        <v/>
-      </c>
-      <c r="AM10" s="46">
-        <f>SUM(AM4:AM9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="T16" s="46">
+        <f>SUM(T4:T15)</f>
+        <v/>
+      </c>
+      <c r="AC16" s="46">
+        <f>SUM(AC4:AC15)</f>
+        <v/>
+      </c>
+      <c r="AD16" s="47">
+        <f>IF(T16=0,"",AC16/T16)</f>
+        <v/>
+      </c>
+      <c r="AL16" s="48">
+        <f>SUM(AL4:AL15)</f>
+        <v/>
+      </c>
+      <c r="AM16" s="46">
+        <f>SUM(AM4:AM15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Fleet basis</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Raw vessels (sum)</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>Fleet (rounded once)</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Market rev/yr (raw sum)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Bali</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C14" s="23">
-        <f>SUMIFS(AN4:AN9,A4:A9,"Bali",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D14" s="49">
-        <f>IF(C14=0,0,CEILING(C14,1))</f>
-        <v/>
-      </c>
-      <c r="E14" s="50">
-        <f>SUMIFS(AO4:AO9,A4:A9,"Bali",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="C20" s="23">
+        <f>SUMIFS(AN4:AN15,A4:A15,"Bali",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D20" s="49">
+        <f>IF(C20=0,0,CEILING(C20,1))</f>
+        <v/>
+      </c>
+      <c r="E20" s="50">
+        <f>SUMIFS(AO4:AO15,A4:A15,"Bali",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Phuket</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C15" s="23">
-        <f>SUMIFS(AN4:AN9,A4:A9,"Phuket",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D15" s="49">
-        <f>IF(C15=0,0,CEILING(C15,1))</f>
-        <v/>
-      </c>
-      <c r="E15" s="50">
-        <f>SUMIFS(AO4:AO9,A4:A9,"Phuket",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="C21" s="23">
+        <f>SUMIFS(AN4:AN15,A4:A15,"Phuket",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D21" s="49">
+        <f>IF(C21=0,0,CEILING(C21,1))</f>
+        <v/>
+      </c>
+      <c r="E21" s="50">
+        <f>SUMIFS(AO4:AO15,A4:A15,"Phuket",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Palm Jumeirah</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>network_sum / ceil</t>
         </is>
       </c>
-      <c r="C16" s="23">
-        <f>SUMIFS(AN4:AN9,A4:A9,"Palm Jumeirah",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="D16" s="49">
-        <f>IF(C16=0,0,CEILING(C16,1))</f>
-        <v/>
-      </c>
-      <c r="E16" s="50">
-        <f>SUMIFS(AO4:AO9,A4:A9,"Palm Jumeirah",AP4:AP9,"=",AQ4:AQ9,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="45" t="inlineStr">
+      <c r="C22" s="23">
+        <f>SUMIFS(AN4:AN15,A4:A15,"Palm Jumeirah",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="D22" s="49">
+        <f>IF(C22=0,0,CEILING(C22,1))</f>
+        <v/>
+      </c>
+      <c r="E22" s="50">
+        <f>SUMIFS(AO4:AO15,A4:A15,"Palm Jumeirah",AP4:AP15,"=",AQ4:AQ15,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
         <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D17" s="48">
-        <f>SUM(D14:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="46">
-        <f>SUM(E14:E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="51" t="inlineStr">
-        <is>
-          <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
-        </is>
-      </c>
-      <c r="C19" s="52" t="inlineStr">
-        <is>
-          <t>Phuket → Langkawi (cross-border, regional reach) (107nm)</t>
-        </is>
+      <c r="D23" s="48">
+        <f>SUM(D20:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="46">
+        <f>SUM(E20:E22)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A18:L18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4076,12 +5243,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="53" t="inlineStr">
+      <c r="A26" s="51" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B26" s="54" t="inlineStr">
+      <c r="B26" s="52" t="inlineStr">
         <is>
           <t>All rungs are one multiplication chain off M_today, which is live off the corridor floor. Change any input (a fare, a multiplier, the scenario) and the whole ladder moves. Bands (low/MID/high) are never single points; greenfield census is per-partner.</t>
         </is>

</xml_diff>